<commit_message>
adding lesson 1.4 practice excersise of skline distribution
</commit_message>
<xml_diff>
--- a/lesson-1-4-visualizing-distributions/bakery_distributions.xlsx
+++ b/lesson-1-4-visualizing-distributions/bakery_distributions.xlsx
@@ -5,7 +5,7 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Lenovo\northstar-coursework\module-01-foundations-of-analytics-and-statistics\lesson-1-4-visualizing-distributions\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Lenovo\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:9_{C0D11222-03C9-4AA4-B4C9-A4DB897119CA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
@@ -18,18 +18,15 @@
   <definedNames>
     <definedName name="_xlchart.v1.0" hidden="1">bakery_distributions!$B$2:$B$51</definedName>
     <definedName name="_xlchart.v1.1" hidden="1">bakery_distributions!$E$1</definedName>
-    <definedName name="_xlchart.v1.10" hidden="1">bakery_distributions!$F$1</definedName>
-    <definedName name="_xlchart.v1.11" hidden="1">bakery_distributions!$F$2:$F$51</definedName>
-    <definedName name="_xlchart.v1.12" hidden="1">bakery_distributions!$F$1</definedName>
-    <definedName name="_xlchart.v1.13" hidden="1">bakery_distributions!$F$2:$F$51</definedName>
+    <definedName name="_xlchart.v1.10" hidden="1">bakery_distributions!$F$2:$F$51</definedName>
     <definedName name="_xlchart.v1.2" hidden="1">bakery_distributions!$E$2:$E$51</definedName>
     <definedName name="_xlchart.v1.3" hidden="1">bakery_distributions!$E$1</definedName>
     <definedName name="_xlchart.v1.4" hidden="1">bakery_distributions!$E$2:$E$51</definedName>
-    <definedName name="_xlchart.v1.5" hidden="1">bakery_distributions!$E$1</definedName>
-    <definedName name="_xlchart.v1.6" hidden="1">bakery_distributions!$E$2:$E$51</definedName>
-    <definedName name="_xlchart.v1.7" hidden="1">bakery_distributions!$B$2:$B$51</definedName>
-    <definedName name="_xlchart.v1.8" hidden="1">bakery_distributions!$E$1</definedName>
-    <definedName name="_xlchart.v1.9" hidden="1">bakery_distributions!$E$2:$E$51</definedName>
+    <definedName name="_xlchart.v1.5" hidden="1">bakery_distributions!$F$1</definedName>
+    <definedName name="_xlchart.v1.6" hidden="1">bakery_distributions!$F$2:$F$51</definedName>
+    <definedName name="_xlchart.v1.7" hidden="1">bakery_distributions!$E$1</definedName>
+    <definedName name="_xlchart.v1.8" hidden="1">bakery_distributions!$E$2:$E$51</definedName>
+    <definedName name="_xlchart.v1.9" hidden="1">bakery_distributions!$F$1</definedName>
   </definedNames>
   <calcPr calcId="0"/>
 </workbook>
@@ -771,28 +768,31 @@
   <cx:chart>
     <cx:title pos="t" align="ctr" overlay="0">
       <cx:tx>
-        <cx:rich>
-          <a:bodyPr spcFirstLastPara="1" vertOverflow="ellipsis" horzOverflow="overflow" wrap="square" lIns="0" tIns="0" rIns="0" bIns="0" anchor="ctr" anchorCtr="1"/>
-          <a:lstStyle/>
-          <a:p>
-            <a:pPr algn="ctr" rtl="0">
-              <a:defRPr/>
-            </a:pPr>
-            <a:r>
-              <a:rPr lang="en-US" sz="1400" b="0" i="0" u="none" strike="noStrike" baseline="0">
-                <a:solidFill>
-                  <a:sysClr val="windowText" lastClr="000000">
-                    <a:lumMod val="65000"/>
-                    <a:lumOff val="35000"/>
-                  </a:sysClr>
-                </a:solidFill>
-                <a:latin typeface="Aptos Narrow" panose="02110004020202020204"/>
-              </a:rPr>
-              <a:t>Distribution of Total Spent (USD)</a:t>
-            </a:r>
-          </a:p>
-        </cx:rich>
+        <cx:txData>
+          <cx:v>Distribution of Total Spent (USD)</cx:v>
+        </cx:txData>
       </cx:tx>
+      <cx:txPr>
+        <a:bodyPr spcFirstLastPara="1" vertOverflow="ellipsis" horzOverflow="overflow" wrap="square" lIns="0" tIns="0" rIns="0" bIns="0" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr algn="ctr" rtl="0">
+            <a:defRPr/>
+          </a:pPr>
+          <a:r>
+            <a:rPr lang="en-US" sz="1400" b="0" i="0" u="none" strike="noStrike" baseline="0">
+              <a:solidFill>
+                <a:sysClr val="windowText" lastClr="000000">
+                  <a:lumMod val="65000"/>
+                  <a:lumOff val="35000"/>
+                </a:sysClr>
+              </a:solidFill>
+              <a:latin typeface="Aptos Narrow" panose="02110004020202020204"/>
+            </a:rPr>
+            <a:t>Distribution of Total Spent (USD)</a:t>
+          </a:r>
+        </a:p>
+      </cx:txPr>
     </cx:title>
     <cx:plotArea>
       <cx:plotAreaRegion>
@@ -886,42 +886,45 @@
   <cx:chartData>
     <cx:data id="0">
       <cx:numDim type="val">
-        <cx:f>_xlchart.v1.11</cx:f>
+        <cx:f>_xlchart.v1.6</cx:f>
       </cx:numDim>
     </cx:data>
   </cx:chartData>
   <cx:chart>
     <cx:title pos="t" align="ctr" overlay="0">
       <cx:tx>
-        <cx:rich>
-          <a:bodyPr spcFirstLastPara="1" vertOverflow="ellipsis" horzOverflow="overflow" wrap="square" lIns="0" tIns="0" rIns="0" bIns="0" anchor="ctr" anchorCtr="1"/>
-          <a:lstStyle/>
-          <a:p>
-            <a:pPr algn="ctr" rtl="0">
-              <a:defRPr/>
-            </a:pPr>
-            <a:r>
-              <a:rPr lang="en-US" sz="1400" b="0" i="0" u="none" strike="noStrike" baseline="0">
-                <a:solidFill>
-                  <a:sysClr val="windowText" lastClr="000000">
-                    <a:lumMod val="65000"/>
-                    <a:lumOff val="35000"/>
-                  </a:sysClr>
-                </a:solidFill>
-                <a:latin typeface="Aptos Narrow" panose="02110004020202020204"/>
-              </a:rPr>
-              <a:t>Distribution of Visit in the Last year</a:t>
-            </a:r>
-          </a:p>
-        </cx:rich>
+        <cx:txData>
+          <cx:v>Distribution of Visit in the Last year</cx:v>
+        </cx:txData>
       </cx:tx>
+      <cx:txPr>
+        <a:bodyPr spcFirstLastPara="1" vertOverflow="ellipsis" horzOverflow="overflow" wrap="square" lIns="0" tIns="0" rIns="0" bIns="0" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr algn="ctr" rtl="0">
+            <a:defRPr/>
+          </a:pPr>
+          <a:r>
+            <a:rPr lang="en-US" sz="1400" b="0" i="0" u="none" strike="noStrike" baseline="0">
+              <a:solidFill>
+                <a:sysClr val="windowText" lastClr="000000">
+                  <a:lumMod val="65000"/>
+                  <a:lumOff val="35000"/>
+                </a:sysClr>
+              </a:solidFill>
+              <a:latin typeface="Aptos Narrow" panose="02110004020202020204"/>
+            </a:rPr>
+            <a:t>Distribution of Visit in the Last year</a:t>
+          </a:r>
+        </a:p>
+      </cx:txPr>
     </cx:title>
     <cx:plotArea>
       <cx:plotAreaRegion>
         <cx:series layoutId="clusteredColumn" uniqueId="{00000000-9E2A-4489-AD88-C8E3086EA27E}">
           <cx:tx>
             <cx:txData>
-              <cx:f>_xlchart.v1.10</cx:f>
+              <cx:f>_xlchart.v1.5</cx:f>
               <cx:v>visits_last_year</cx:v>
             </cx:txData>
           </cx:tx>
@@ -1008,7 +1011,7 @@
   <cx:chartData>
     <cx:data id="0">
       <cx:numDim type="val">
-        <cx:f>_xlchart.v1.6</cx:f>
+        <cx:f>_xlchart.v1.8</cx:f>
       </cx:numDim>
     </cx:data>
   </cx:chartData>
@@ -1046,7 +1049,7 @@
         <cx:series layoutId="boxWhisker" uniqueId="{00000000-F278-434E-AD99-828931351232}">
           <cx:tx>
             <cx:txData>
-              <cx:f>_xlchart.v1.5</cx:f>
+              <cx:f>_xlchart.v1.7</cx:f>
               <cx:v>total_spent_usd</cx:v>
             </cx:txData>
           </cx:tx>
@@ -1124,7 +1127,7 @@
   <cx:chartData>
     <cx:data id="0">
       <cx:numDim type="val">
-        <cx:f>_xlchart.v1.13</cx:f>
+        <cx:f>_xlchart.v1.10</cx:f>
       </cx:numDim>
     </cx:data>
   </cx:chartData>
@@ -1162,7 +1165,7 @@
         <cx:series layoutId="boxWhisker" uniqueId="{00000000-5AFA-46F0-83EE-B20470EC5876}">
           <cx:tx>
             <cx:txData>
-              <cx:f>_xlchart.v1.12</cx:f>
+              <cx:f>_xlchart.v1.9</cx:f>
               <cx:v>visits_last_year</cx:v>
             </cx:txData>
           </cx:tx>
@@ -1220,10 +1223,10 @@
   <cx:chartData>
     <cx:data id="0">
       <cx:strDim type="cat">
-        <cx:f>_xlchart.v1.7</cx:f>
+        <cx:f>_xlchart.v1.0</cx:f>
       </cx:strDim>
       <cx:numDim type="val">
-        <cx:f>_xlchart.v1.9</cx:f>
+        <cx:f>_xlchart.v1.2</cx:f>
       </cx:numDim>
     </cx:data>
   </cx:chartData>
@@ -1261,7 +1264,7 @@
         <cx:series layoutId="boxWhisker" uniqueId="{00000000-FA08-4B2B-9BE0-3AE884C4C6B7}">
           <cx:tx>
             <cx:txData>
-              <cx:f>_xlchart.v1.8</cx:f>
+              <cx:f>_xlchart.v1.1</cx:f>
               <cx:v>total_spent_usd</cx:v>
             </cx:txData>
           </cx:tx>
@@ -4203,8 +4206,8 @@
           </xdr:nvSpPr>
           <xdr:spPr>
             <a:xfrm>
-              <a:off x="5474757" y="5320685"/>
-              <a:ext cx="6160082" cy="4163962"/>
+              <a:off x="5476874" y="5314950"/>
+              <a:ext cx="6181112" cy="4159250"/>
             </a:xfrm>
             <a:prstGeom prst="rect">
               <a:avLst/>
@@ -4359,8 +4362,8 @@
           </xdr:nvSpPr>
           <xdr:spPr>
             <a:xfrm>
-              <a:off x="11974837" y="5329550"/>
-              <a:ext cx="5272581" cy="4195449"/>
+              <a:off x="11997984" y="5323815"/>
+              <a:ext cx="5289787" cy="4190737"/>
             </a:xfrm>
             <a:prstGeom prst="rect">
               <a:avLst/>
@@ -4437,8 +4440,8 @@
           </xdr:nvSpPr>
           <xdr:spPr>
             <a:xfrm>
-              <a:off x="5480801" y="9986706"/>
-              <a:ext cx="6078929" cy="3962810"/>
+              <a:off x="5484829" y="9975645"/>
+              <a:ext cx="6098048" cy="3958508"/>
             </a:xfrm>
             <a:prstGeom prst="rect">
               <a:avLst/>

</xml_diff>